<commit_message>
feat(slot): console sample game, Unity implementation, docs and CI
- samples/ConsoleSlot: terminal slot on the SDK (interactive + --demo)
- unity/: Unity 6 project built on unity-claude-starter; SDK referenced as
  a local UPM package. Procedural UI/sprites/SFX, splice-based reel stops
  (ReelMotion), anticipation, win tiers, free spins, save/resume,
  auto-created Main scene. EditMode/PlayMode tests.
- Unity C# compile-checked against reference DLLs; not yet run in the
  Unity Editor (documented in README)
- README/CLAUDE.md for slot-project, CI workflow for SDK + math checks

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FMGeisuxnqEQV9jERtZ16C
</commit_message>
<xml_diff>
--- a/slot-project/docs/game_spec.xlsx
+++ b/slot-project/docs/game_spec.xlsx
@@ -407,7 +407,7 @@
     <t xml:space="preserve">Message bar</t>
   </si>
   <si>
-    <t xml:space="preserve">(0, -300) 1164x56</t>
+    <t xml:space="preserve">(0, -318) 1164x56</t>
   </si>
   <si>
     <t xml:space="preserve">Idle: GOOD LUCK / on a win: line details / FS: messages</t>
@@ -647,7 +647,7 @@
     <t xml:space="preserve">→ S1</t>
   </si>
   <si>
-    <t xml:space="preserve">Auto play stop conditions: AUTO pressed again / insufficient balance / BIG WIN or above / free spins triggered (auto continues after FS ends)</t>
+    <t xml:space="preserve">Auto play stop conditions: AUTO pressed again / insufficient balance / BIG WIN or above in the base game. When free spins trigger, the FS play automatically and auto play resumes after they end.</t>
   </si>
   <si>
     <t xml:space="preserve">Control</t>

</xml_diff>